<commit_message>
Fix ASL interpreters showing blank languages
</commit_message>
<xml_diff>
--- a/active_linguists_2026.xlsx
+++ b/active_linguists_2026.xlsx
@@ -537,7 +537,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Albanian, Arabic, Bengali, Burmese, Chinese - Mandarin, Chinese - Traditional, DTP, DTP(Word)_Pashto, DTP(Word)_Persian, Dari, English, Haitian Creole, Haitian_Creole, Hmong, Italian, Karen, Lao, Mandarin Chinese, Norwegian, Pashto, Persian, Polish, Portuguese, Spanish, Spanish_Doc-Trans, Swedish, Vietnamese</t>
+          <t>ASL, Albanian, Arabic, Bengali, Burmese, Chinese - Mandarin, Chinese - Traditional, DTP, DTP(Word)_Pashto, DTP(Word)_Persian, Dari, English, Haitian Creole, Haitian_Creole, Hmong, Italian, Karen, Lao, Mandarin Chinese, Norwegian, Pashto, Persian, Polish, Portuguese, Spanish, Spanish_Doc-Trans, Swedish, Vietnamese</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
@@ -760,7 +760,11 @@
           <t>terpdarci@gmail.com</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D13" s="3" t="n">
         <v>32</v>
       </c>
@@ -1406,7 +1410,11 @@
           <t>dawnterp76@gmail.com</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D39" s="3" t="n">
         <v>11</v>
       </c>
@@ -1802,7 +1810,11 @@
           <t>swiftcrimson18@yahoo.com</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr"/>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D55" s="3" t="n">
         <v>7</v>
       </c>
@@ -2848,7 +2860,11 @@
           <t>marciamarshall@outlook.com</t>
         </is>
       </c>
-      <c r="C97" s="2" t="inlineStr"/>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D97" s="3" t="n">
         <v>3</v>
       </c>
@@ -2894,7 +2910,11 @@
           <t>cejfalter@hotmail.com</t>
         </is>
       </c>
-      <c r="C99" s="2" t="inlineStr"/>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D99" s="3" t="n">
         <v>3</v>
       </c>
@@ -3015,7 +3035,11 @@
           <t>escinaw10101@gmail.com</t>
         </is>
       </c>
-      <c r="C104" s="2" t="inlineStr"/>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D104" s="3" t="n">
         <v>3</v>
       </c>
@@ -4286,7 +4310,11 @@
           <t>candice.barrier@gmail.com</t>
         </is>
       </c>
-      <c r="C155" s="2" t="inlineStr"/>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D155" s="3" t="n">
         <v>2</v>
       </c>
@@ -7528,7 +7556,11 @@
           <t>ashleycbarbour@gmail.com</t>
         </is>
       </c>
-      <c r="C285" s="2" t="inlineStr"/>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D285" s="3" t="n">
         <v>1</v>
       </c>
@@ -7649,7 +7681,11 @@
           <t>jatherton8505@gmail.com</t>
         </is>
       </c>
-      <c r="C290" s="2" t="inlineStr"/>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D290" s="3" t="n">
         <v>1</v>
       </c>
@@ -7741,7 +7777,11 @@
           <t>terpharrison@gmail.com</t>
         </is>
       </c>
-      <c r="C294" s="2" t="inlineStr"/>
+      <c r="C294" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D294" s="3" t="n">
         <v>1</v>
       </c>
@@ -7862,7 +7902,11 @@
           <t>CARMENMJ@PRODIGY.NET</t>
         </is>
       </c>
-      <c r="C299" s="2" t="inlineStr"/>
+      <c r="C299" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D299" s="3" t="n">
         <v>1</v>
       </c>
@@ -8175,7 +8219,11 @@
           <t>SonjaSignsASL@gmail.com</t>
         </is>
       </c>
-      <c r="C312" s="2" t="inlineStr"/>
+      <c r="C312" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D312" s="3" t="n">
         <v>1</v>
       </c>
@@ -8196,7 +8244,11 @@
           <t>amandahosek@gmail.com</t>
         </is>
       </c>
-      <c r="C313" s="2" t="inlineStr"/>
+      <c r="C313" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D313" s="3" t="n">
         <v>1</v>
       </c>
@@ -8317,7 +8369,11 @@
           <t>nowickifam@gmail.com</t>
         </is>
       </c>
-      <c r="C318" s="2" t="inlineStr"/>
+      <c r="C318" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D318" s="3" t="n">
         <v>1</v>
       </c>
@@ -8338,7 +8394,11 @@
           <t>driddick53@gmail.com</t>
         </is>
       </c>
-      <c r="C319" s="2" t="inlineStr"/>
+      <c r="C319" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D319" s="3" t="n">
         <v>1</v>
       </c>
@@ -8359,7 +8419,11 @@
           <t>ethelpeiffer@gmail.com</t>
         </is>
       </c>
-      <c r="C320" s="2" t="inlineStr"/>
+      <c r="C320" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D320" s="3" t="n">
         <v>1</v>
       </c>
@@ -8380,7 +8444,11 @@
           <t>jenniferp78@yahoo.com</t>
         </is>
       </c>
-      <c r="C321" s="2" t="inlineStr"/>
+      <c r="C321" s="2" t="inlineStr">
+        <is>
+          <t>ASL</t>
+        </is>
+      </c>
       <c r="D321" s="3" t="n">
         <v>1</v>
       </c>

</xml_diff>